<commit_message>
Table finished as discussed until now.
</commit_message>
<xml_diff>
--- a/data/manual/all_unique_materials_commodities.xlsx
+++ b/data/manual/all_unique_materials_commodities.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B49"/>
+  <dimension ref="A1:B50"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -755,11 +755,7 @@
       <c r="A34" s="1" t="n">
         <v>32</v>
       </c>
-      <c r="B34" t="inlineStr">
-        <is>
-          <t>PGM</t>
-        </is>
-      </c>
+      <c r="B34" t="inlineStr"/>
     </row>
     <row r="35">
       <c r="A35" s="1" t="n">
@@ -767,7 +763,7 @@
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>Cobalt</t>
+          <t>PGM</t>
         </is>
       </c>
     </row>
@@ -777,7 +773,7 @@
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>Nickel</t>
+          <t>Cobalt</t>
         </is>
       </c>
     </row>
@@ -787,7 +783,7 @@
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>Phosphate and Phosphorus oxides</t>
+          <t>Nickel</t>
         </is>
       </c>
     </row>
@@ -797,7 +793,7 @@
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>Diamonds (unspecified)</t>
+          <t>Phosphate and Phosphorus oxides</t>
         </is>
       </c>
     </row>
@@ -807,7 +803,7 @@
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>Manganese</t>
+          <t>Diamonds (unspecified)</t>
         </is>
       </c>
     </row>
@@ -817,7 +813,7 @@
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>Lead</t>
+          <t>Manganese</t>
         </is>
       </c>
     </row>
@@ -827,7 +823,7 @@
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>Niobium</t>
+          <t>Lead</t>
         </is>
       </c>
     </row>
@@ -837,7 +833,7 @@
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>Ilmenite</t>
+          <t>Niobium</t>
         </is>
       </c>
     </row>
@@ -847,7 +843,7 @@
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>Rutile</t>
+          <t>Ilmenite</t>
         </is>
       </c>
     </row>
@@ -857,7 +853,7 @@
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>Zircon</t>
+          <t>Rutile</t>
         </is>
       </c>
     </row>
@@ -867,7 +863,7 @@
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>Palladium</t>
+          <t>Zircon</t>
         </is>
       </c>
     </row>
@@ -877,7 +873,7 @@
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>Platinum</t>
+          <t>Palladium</t>
         </is>
       </c>
     </row>
@@ -887,7 +883,7 @@
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>Lithium oxide</t>
+          <t>Platinum</t>
         </is>
       </c>
     </row>
@@ -897,7 +893,7 @@
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>Tin</t>
+          <t>Lithium oxide</t>
         </is>
       </c>
     </row>
@@ -906,6 +902,16 @@
         <v>47</v>
       </c>
       <c r="B49" t="inlineStr">
+        <is>
+          <t>Tin</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="1" t="n">
+        <v>48</v>
+      </c>
+      <c r="B50" t="inlineStr">
         <is>
           <t>Tellurium</t>
         </is>

</xml_diff>